<commit_message>
Publish Duisburg_2011_WC, Poznan_2011_WC, Szeged_2011_WCH
</commit_message>
<xml_diff>
--- a/events/Duisburg_2011_WC/Duisburg_2011_WC_Results.xlsx
+++ b/events/Duisburg_2011_WC/Duisburg_2011_WC_Results.xlsx
@@ -3443,6 +3443,11 @@
           <t>1:59.304</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>47909</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14975,6 +14980,11 @@
           <t>2:03.570</t>
         </is>
       </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>47909</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -56004,6 +56014,11 @@
           <t>73492</t>
         </is>
       </c>
+      <c r="S860" t="inlineStr">
+        <is>
+          <t>47909</t>
+        </is>
+      </c>
     </row>
     <row r="861">
       <c r="A861" t="inlineStr">
@@ -68563,6 +68578,11 @@
           <t>73492</t>
         </is>
       </c>
+      <c r="S1057" t="inlineStr">
+        <is>
+          <t>47909</t>
+        </is>
+      </c>
     </row>
     <row r="1058">
       <c r="A1058" t="inlineStr">
@@ -76674,6 +76694,11 @@
       <c r="R1182" t="inlineStr">
         <is>
           <t>73492</t>
+        </is>
+      </c>
+      <c r="S1182" t="inlineStr">
+        <is>
+          <t>47909</t>
         </is>
       </c>
     </row>
@@ -92120,7 +92145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D253"/>
+  <dimension ref="A1:D254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -97689,6 +97714,28 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>47909</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Alexandra Borbala</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>KEREZTESI</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>